<commit_message>
Fixed bug in sensitivity of stress failure factor
</commit_message>
<xml_diff>
--- a/DataConstantTemperature/3Materials.xlsx
+++ b/DataConstantTemperature/3Materials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataConstantTemperature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnan Suresh\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataConstantTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBD3386-E784-4D12-8B64-5FC06A88FEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56AD1F71-3634-4D72-9A06-E97FADD31182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="24375" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
   <si>
     <t>Attribute</t>
   </si>
@@ -98,19 +98,13 @@
   </si>
   <si>
     <t>7068 Al</t>
-  </si>
-  <si>
-    <t>Criticality</t>
-  </si>
-  <si>
-    <t>Dimensionless</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,14 +115,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -170,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -179,9 +165,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -470,15 +453,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
-    <col min="2" max="702" width="20.5546875" style="1" customWidth="1"/>
-    <col min="703" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="1" customWidth="1"/>
+    <col min="5" max="700" width="20.5703125" style="1" customWidth="1"/>
+    <col min="701" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -489,16 +475,10 @@
         <v>5</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>20</v>
       </c>
@@ -509,73 +489,49 @@
         <v>12</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <v>7850</v>
       </c>
-      <c r="C3" s="6">
-        <v>2.1</v>
+      <c r="C3" s="5">
+        <v>210000000000</v>
       </c>
       <c r="D3" s="5">
-        <v>6</v>
-      </c>
-      <c r="E3" s="6">
         <v>250000000</v>
       </c>
-      <c r="F3" s="5">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <v>7800</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>200000000000</v>
       </c>
       <c r="D4" s="5">
-        <v>4</v>
-      </c>
-      <c r="E4" s="6">
-        <v>200000000</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+        <v>180000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>2700</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>70000000000</v>
       </c>
       <c r="D5" s="5">
-        <v>2</v>
-      </c>
-      <c r="E5" s="6">
         <v>100000000</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -603,12 +559,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC80EBF-8B96-4896-8C13-AD8A976D05A3}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -622,7 +578,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -636,7 +592,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -650,7 +606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -664,7 +620,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>

</xml_diff>